<commit_message>
G2: MPS χ=128 submission, scored 498/600
problems/05_graded_G2/mps_chi128_values.csv: the uploaded G2_v1 values (MPS,
bond dimension 128, BlueQubit mps.cpu, 0 credits). Scored 498/600 (corr² ≈ 0.83).
README records the method, why MPS/χ=128 was chosen (S2 and a local G2-shaped
test chain reached corr² 1.00), and why it is short of 100%: χ=128 is not
converged on the 36-qubit chain (χ=256 moved values by up to 0.06), and χ=256
for the remaining qubits is estimated at ~$10.88 per job.
runs/ledger.csv, runs/hidden_2.xlsx: G2 job records.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/runs/hidden_2.xlsx
+++ b/runs/hidden_2.xlsx
@@ -7,6 +7,7 @@
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimates" sheetId="3" r:id="R5ebadaf271a24139"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jobs" sheetId="4" r:id="Rd12004dcc1cd4dcf"/>
   </x:sheets>
+  <x:calcPr fullCalcOnLoad="1"/>
 </x:workbook>
 </file>
 
@@ -467,7 +468,11 @@
       <x:c r="A4" s="2" t="str">
         <x:v>Official circuit ID</x:v>
       </x:c>
-      <x:c r="B4" s="6"/>
+      <x:c r="B4" s="6" t="inlineStr">
+        <x:is>
+          <x:t>G2</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C4" s="2"/>
       <x:c r="D4" s="10" t="str">
         <x:v>Precision settings</x:v>
@@ -487,7 +492,9 @@
       <x:c r="A5" s="2" t="str">
         <x:v>Required qubits</x:v>
       </x:c>
-      <x:c r="B5" s="6"/>
+      <x:c r="B5" s="6" t="n">
+        <x:v>36</x:v>
+      </x:c>
       <x:c r="C5" s="2"/>
       <x:c r="D5" s="2" t="str">
         <x:v>MPS bond dimension χ</x:v>
@@ -1124,7 +1131,9 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="21"/>
+      <x:c r="A6" s="21" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="B6" s="19"/>
       <x:c r="C6" s="13" t="str">
         <x:f>IF(OR(COUNTA($A6)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A6,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A6,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A6,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A6,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -1180,7 +1189,9 @@
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="21"/>
+      <x:c r="A7" s="21" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="B7" s="19"/>
       <x:c r="C7" s="13" t="str">
         <x:f>IF(OR(COUNTA($A7)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A7,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A7,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A7,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A7,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -1236,7 +1247,9 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="21"/>
+      <x:c r="A8" s="21" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="B8" s="19"/>
       <x:c r="C8" s="13" t="str">
         <x:f>IF(OR(COUNTA($A8)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A8,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A8,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A8,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A8,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -1292,7 +1305,9 @@
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="21"/>
+      <x:c r="A9" s="21" t="n">
+        <x:v>3</x:v>
+      </x:c>
       <x:c r="B9" s="19"/>
       <x:c r="C9" s="13" t="str">
         <x:f>IF(OR(COUNTA($A9)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A9,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A9,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A9,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A9,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -1348,7 +1363,9 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="21"/>
+      <x:c r="A10" s="21" t="n">
+        <x:v>4</x:v>
+      </x:c>
       <x:c r="B10" s="19"/>
       <x:c r="C10" s="13" t="str">
         <x:f>IF(OR(COUNTA($A10)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A10,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A10,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A10,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A10,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -1404,7 +1421,9 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="21"/>
+      <x:c r="A11" s="21" t="n">
+        <x:v>5</x:v>
+      </x:c>
       <x:c r="B11" s="19"/>
       <x:c r="C11" s="13" t="str">
         <x:f>IF(OR(COUNTA($A11)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A11,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A11,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A11,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A11,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -1460,7 +1479,9 @@
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="21"/>
+      <x:c r="A12" s="21" t="n">
+        <x:v>6</x:v>
+      </x:c>
       <x:c r="B12" s="19"/>
       <x:c r="C12" s="13" t="str">
         <x:f>IF(OR(COUNTA($A12)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A12,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A12,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A12,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A12,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -1516,7 +1537,9 @@
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="21"/>
+      <x:c r="A13" s="21" t="n">
+        <x:v>7</x:v>
+      </x:c>
       <x:c r="B13" s="19"/>
       <x:c r="C13" s="13" t="str">
         <x:f>IF(OR(COUNTA($A13)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A13,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A13,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A13,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A13,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -1572,7 +1595,9 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="21"/>
+      <x:c r="A14" s="21" t="n">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="B14" s="19"/>
       <x:c r="C14" s="13" t="str">
         <x:f>IF(OR(COUNTA($A14)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A14,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A14,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A14,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A14,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -1628,7 +1653,9 @@
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="21"/>
+      <x:c r="A15" s="21" t="n">
+        <x:v>9</x:v>
+      </x:c>
       <x:c r="B15" s="19"/>
       <x:c r="C15" s="13" t="str">
         <x:f>IF(OR(COUNTA($A15)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A15,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A15,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A15,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A15,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -1684,7 +1711,9 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="21"/>
+      <x:c r="A16" s="21" t="n">
+        <x:v>10</x:v>
+      </x:c>
       <x:c r="B16" s="19"/>
       <x:c r="C16" s="13" t="str">
         <x:f>IF(OR(COUNTA($A16)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A16,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A16,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A16,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A16,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -1740,7 +1769,9 @@
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="21"/>
+      <x:c r="A17" s="21" t="n">
+        <x:v>11</x:v>
+      </x:c>
       <x:c r="B17" s="19"/>
       <x:c r="C17" s="13" t="str">
         <x:f>IF(OR(COUNTA($A17)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A17,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A17,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A17,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A17,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -1796,7 +1827,9 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="21"/>
+      <x:c r="A18" s="21" t="n">
+        <x:v>12</x:v>
+      </x:c>
       <x:c r="B18" s="19"/>
       <x:c r="C18" s="13" t="str">
         <x:f>IF(OR(COUNTA($A18)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A18,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A18,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A18,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A18,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -1852,7 +1885,9 @@
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="21"/>
+      <x:c r="A19" s="21" t="n">
+        <x:v>13</x:v>
+      </x:c>
       <x:c r="B19" s="19"/>
       <x:c r="C19" s="13" t="str">
         <x:f>IF(OR(COUNTA($A19)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A19,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A19,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A19,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A19,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -1908,7 +1943,9 @@
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="21"/>
+      <x:c r="A20" s="21" t="n">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="B20" s="19"/>
       <x:c r="C20" s="13" t="str">
         <x:f>IF(OR(COUNTA($A20)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A20,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A20,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A20,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A20,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -1964,7 +2001,9 @@
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="21"/>
+      <x:c r="A21" s="21" t="n">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="B21" s="19"/>
       <x:c r="C21" s="13" t="str">
         <x:f>IF(OR(COUNTA($A21)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A21,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A21,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A21,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A21,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -2020,7 +2059,9 @@
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="21"/>
+      <x:c r="A22" s="21" t="n">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="B22" s="19"/>
       <x:c r="C22" s="13" t="str">
         <x:f>IF(OR(COUNTA($A22)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A22,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A22,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A22,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A22,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -2076,7 +2117,9 @@
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="21"/>
+      <x:c r="A23" s="21" t="n">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="B23" s="19"/>
       <x:c r="C23" s="13" t="str">
         <x:f>IF(OR(COUNTA($A23)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A23,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A23,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A23,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A23,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -2132,7 +2175,9 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="21"/>
+      <x:c r="A24" s="21" t="n">
+        <x:v>18</x:v>
+      </x:c>
       <x:c r="B24" s="19"/>
       <x:c r="C24" s="13" t="str">
         <x:f>IF(OR(COUNTA($A24)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A24,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A24,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A24,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A24,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -2188,7 +2233,9 @@
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="21"/>
+      <x:c r="A25" s="21" t="n">
+        <x:v>19</x:v>
+      </x:c>
       <x:c r="B25" s="19"/>
       <x:c r="C25" s="13" t="str">
         <x:f>IF(OR(COUNTA($A25)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A25,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A25,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A25,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A25,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -2244,7 +2291,9 @@
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="21"/>
+      <x:c r="A26" s="21" t="n">
+        <x:v>20</x:v>
+      </x:c>
       <x:c r="B26" s="19"/>
       <x:c r="C26" s="13" t="str">
         <x:f>IF(OR(COUNTA($A26)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A26,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A26,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A26,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A26,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -2300,7 +2349,9 @@
       </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="21"/>
+      <x:c r="A27" s="21" t="n">
+        <x:v>21</x:v>
+      </x:c>
       <x:c r="B27" s="19"/>
       <x:c r="C27" s="13" t="str">
         <x:f>IF(OR(COUNTA($A27)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A27,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A27,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A27,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A27,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -2356,7 +2407,9 @@
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="21"/>
+      <x:c r="A28" s="21" t="n">
+        <x:v>22</x:v>
+      </x:c>
       <x:c r="B28" s="19"/>
       <x:c r="C28" s="13" t="str">
         <x:f>IF(OR(COUNTA($A28)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A28,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A28,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A28,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A28,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -2412,7 +2465,9 @@
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="21"/>
+      <x:c r="A29" s="21" t="n">
+        <x:v>23</x:v>
+      </x:c>
       <x:c r="B29" s="19"/>
       <x:c r="C29" s="13" t="str">
         <x:f>IF(OR(COUNTA($A29)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A29,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A29,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A29,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A29,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -2468,7 +2523,9 @@
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="21"/>
+      <x:c r="A30" s="21" t="n">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="B30" s="19"/>
       <x:c r="C30" s="13" t="str">
         <x:f>IF(OR(COUNTA($A30)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A30,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A30,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A30,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A30,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -2524,7 +2581,9 @@
       </x:c>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="21"/>
+      <x:c r="A31" s="21" t="n">
+        <x:v>25</x:v>
+      </x:c>
       <x:c r="B31" s="19"/>
       <x:c r="C31" s="13" t="str">
         <x:f>IF(OR(COUNTA($A31)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A31,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A31,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A31,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A31,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -2580,7 +2639,9 @@
       </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="21"/>
+      <x:c r="A32" s="21" t="n">
+        <x:v>26</x:v>
+      </x:c>
       <x:c r="B32" s="19"/>
       <x:c r="C32" s="13" t="str">
         <x:f>IF(OR(COUNTA($A32)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A32,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A32,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A32,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A32,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -2636,7 +2697,9 @@
       </x:c>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="21"/>
+      <x:c r="A33" s="21" t="n">
+        <x:v>27</x:v>
+      </x:c>
       <x:c r="B33" s="19"/>
       <x:c r="C33" s="13" t="str">
         <x:f>IF(OR(COUNTA($A33)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A33,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A33,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A33,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A33,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -2692,7 +2755,9 @@
       </x:c>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="21"/>
+      <x:c r="A34" s="21" t="n">
+        <x:v>28</x:v>
+      </x:c>
       <x:c r="B34" s="19"/>
       <x:c r="C34" s="13" t="str">
         <x:f>IF(OR(COUNTA($A34)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A34,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A34,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A34,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A34,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -2748,7 +2813,9 @@
       </x:c>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="21"/>
+      <x:c r="A35" s="21" t="n">
+        <x:v>29</x:v>
+      </x:c>
       <x:c r="B35" s="19"/>
       <x:c r="C35" s="13" t="str">
         <x:f>IF(OR(COUNTA($A35)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A35,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A35,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A35,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A35,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -2804,7 +2871,9 @@
       </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="21"/>
+      <x:c r="A36" s="21" t="n">
+        <x:v>30</x:v>
+      </x:c>
       <x:c r="B36" s="19"/>
       <x:c r="C36" s="13" t="str">
         <x:f>IF(OR(COUNTA($A36)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A36,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A36,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A36,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A36,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -2860,7 +2929,9 @@
       </x:c>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="21"/>
+      <x:c r="A37" s="21" t="n">
+        <x:v>31</x:v>
+      </x:c>
       <x:c r="B37" s="19"/>
       <x:c r="C37" s="13" t="str">
         <x:f>IF(OR(COUNTA($A37)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A37,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A37,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A37,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A37,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -2916,7 +2987,9 @@
       </x:c>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="21"/>
+      <x:c r="A38" s="21" t="n">
+        <x:v>32</x:v>
+      </x:c>
       <x:c r="B38" s="19"/>
       <x:c r="C38" s="13" t="str">
         <x:f>IF(OR(COUNTA($A38)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A38,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A38,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A38,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A38,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -2972,7 +3045,9 @@
       </x:c>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="21"/>
+      <x:c r="A39" s="21" t="n">
+        <x:v>33</x:v>
+      </x:c>
       <x:c r="B39" s="19"/>
       <x:c r="C39" s="13" t="str">
         <x:f>IF(OR(COUNTA($A39)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A39,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A39,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A39,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A39,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -3028,7 +3103,9 @@
       </x:c>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="21"/>
+      <x:c r="A40" s="21" t="n">
+        <x:v>34</x:v>
+      </x:c>
       <x:c r="B40" s="19"/>
       <x:c r="C40" s="13" t="str">
         <x:f>IF(OR(COUNTA($A40)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A40,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A40,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A40,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A40,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -3084,7 +3161,9 @@
       </x:c>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="21"/>
+      <x:c r="A41" s="21" t="n">
+        <x:v>35</x:v>
+      </x:c>
       <x:c r="B41" s="19"/>
       <x:c r="C41" s="13" t="str">
         <x:f>IF(OR(COUNTA($A41)=0,NOT(ISNUMBER('Status'!$E$5))),"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A41,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)=0,"",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A41,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)&gt;1,"DUP",IF(COUNTIFS('Estimates'!$A$5:$A$2004,$A41,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1,'Estimates'!$F$5:$F$2004,"&lt;&gt;")=0,"",SUMIFS('Estimates'!$F$5:$F$2004,'Estimates'!$A$5:$A$2004,$A41,'Estimates'!$B$5:$B$2004,"MPS",'Estimates'!$C$5:$C$2004,'Status'!$E$5,'Estimates'!$H$5:$H$2004,1)))))</x:f>
@@ -10172,256 +10251,1018 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="6"/>
-      <x:c r="B5" s="6"/>
-      <x:c r="C5" s="6"/>
+      <x:c r="A5" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C5" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D5" s="11"/>
       <x:c r="E5" s="6"/>
-      <x:c r="F5" s="20"/>
-      <x:c r="G5" s="6"/>
-      <x:c r="H5" s="6"/>
+      <x:c r="F5" s="20" t="n">
+        <x:v>0.9969978919142036</x:v>
+      </x:c>
+      <x:c r="G5" s="6" t="inlineStr">
+        <x:is>
+          <x:t>3vthFykOUg9STpyH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H5" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="6"/>
-      <x:c r="B6" s="6"/>
-      <x:c r="C6" s="6"/>
+      <x:c r="A6" s="6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C6" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D6" s="11"/>
       <x:c r="E6" s="6"/>
-      <x:c r="F6" s="20"/>
-      <x:c r="G6" s="6"/>
-      <x:c r="H6" s="6"/>
+      <x:c r="F6" s="20" t="n">
+        <x:v>0.948333185562568</x:v>
+      </x:c>
+      <x:c r="G6" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Yxrh3L2PUkc3VhaY</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H6" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="6"/>
-      <x:c r="B7" s="6"/>
-      <x:c r="C7" s="6"/>
+      <x:c r="A7" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C7" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D7" s="11"/>
       <x:c r="E7" s="6"/>
-      <x:c r="F7" s="20"/>
-      <x:c r="G7" s="6"/>
-      <x:c r="H7" s="6"/>
+      <x:c r="F7" s="20" t="n">
+        <x:v>0.9938676258728648</x:v>
+      </x:c>
+      <x:c r="G7" s="6" t="inlineStr">
+        <x:is>
+          <x:t>amYn6eEGELs0f07u</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H7" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="6"/>
-      <x:c r="B8" s="6"/>
-      <x:c r="C8" s="6"/>
+      <x:c r="A8" s="6" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C8" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D8" s="11"/>
       <x:c r="E8" s="6"/>
-      <x:c r="F8" s="20"/>
-      <x:c r="G8" s="6"/>
-      <x:c r="H8" s="6"/>
+      <x:c r="F8" s="20" t="n">
+        <x:v>0.9156574099163179</x:v>
+      </x:c>
+      <x:c r="G8" s="6" t="inlineStr">
+        <x:is>
+          <x:t>CcP073uy8VTfOm7Z</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H8" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="6"/>
-      <x:c r="B9" s="6"/>
-      <x:c r="C9" s="6"/>
+      <x:c r="A9" s="6" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C9" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D9" s="11"/>
       <x:c r="E9" s="6"/>
-      <x:c r="F9" s="20"/>
-      <x:c r="G9" s="6"/>
-      <x:c r="H9" s="6"/>
+      <x:c r="F9" s="20" t="n">
+        <x:v>0.6244706855017967</x:v>
+      </x:c>
+      <x:c r="G9" s="6" t="inlineStr">
+        <x:is>
+          <x:t>naxElkaIO19i9Z0B</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H9" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="6"/>
-      <x:c r="B10" s="6"/>
-      <x:c r="C10" s="6"/>
+      <x:c r="A10" s="6" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B10" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C10" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D10" s="11"/>
       <x:c r="E10" s="6"/>
-      <x:c r="F10" s="20"/>
-      <x:c r="G10" s="6"/>
-      <x:c r="H10" s="6"/>
+      <x:c r="F10" s="20" t="n">
+        <x:v>0.7307280908829952</x:v>
+      </x:c>
+      <x:c r="G10" s="6" t="inlineStr">
+        <x:is>
+          <x:t>culHIrNwFvzVmhin</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H10" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="6"/>
-      <x:c r="B11" s="6"/>
-      <x:c r="C11" s="6"/>
+      <x:c r="A11" s="6" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B11" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C11" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D11" s="11"/>
       <x:c r="E11" s="6"/>
-      <x:c r="F11" s="20"/>
-      <x:c r="G11" s="6"/>
-      <x:c r="H11" s="6"/>
+      <x:c r="F11" s="20" t="n">
+        <x:v>0.4007412478551923</x:v>
+      </x:c>
+      <x:c r="G11" s="6" t="inlineStr">
+        <x:is>
+          <x:t>B4ds8Aiw7rfVMwe3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H11" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="6"/>
-      <x:c r="B12" s="6"/>
-      <x:c r="C12" s="6"/>
+      <x:c r="A12" s="6" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B12" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D12" s="11"/>
       <x:c r="E12" s="6"/>
-      <x:c r="F12" s="20"/>
-      <x:c r="G12" s="6"/>
-      <x:c r="H12" s="6"/>
+      <x:c r="F12" s="20" t="n">
+        <x:v>0.41734522035241306</x:v>
+      </x:c>
+      <x:c r="G12" s="6" t="inlineStr">
+        <x:is>
+          <x:t>cMCDoXnvsIcrGYIL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H12" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="6"/>
-      <x:c r="B13" s="6"/>
-      <x:c r="C13" s="6"/>
+      <x:c r="A13" s="6" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C13" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D13" s="11"/>
       <x:c r="E13" s="6"/>
-      <x:c r="F13" s="20"/>
-      <x:c r="G13" s="6"/>
-      <x:c r="H13" s="6"/>
+      <x:c r="F13" s="20" t="n">
+        <x:v>0.10835526790114147</x:v>
+      </x:c>
+      <x:c r="G13" s="6" t="inlineStr">
+        <x:is>
+          <x:t>iqlVmKsTe1h6oCoX</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H13" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="6"/>
-      <x:c r="B14" s="6"/>
-      <x:c r="C14" s="6"/>
+      <x:c r="A14" s="6" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B14" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D14" s="11"/>
       <x:c r="E14" s="6"/>
-      <x:c r="F14" s="20"/>
-      <x:c r="G14" s="6"/>
-      <x:c r="H14" s="6"/>
+      <x:c r="F14" s="20" t="n">
+        <x:v>0.10315235933202012</x:v>
+      </x:c>
+      <x:c r="G14" s="6" t="inlineStr">
+        <x:is>
+          <x:t>ddxYjwvqBs0JhZtJ</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H14" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="6"/>
-      <x:c r="B15" s="6"/>
-      <x:c r="C15" s="6"/>
+      <x:c r="A15" s="6" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B15" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C15" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D15" s="11"/>
       <x:c r="E15" s="6"/>
-      <x:c r="F15" s="20"/>
-      <x:c r="G15" s="6"/>
-      <x:c r="H15" s="6"/>
+      <x:c r="F15" s="20" t="n">
+        <x:v>0.1064606618021046</x:v>
+      </x:c>
+      <x:c r="G15" s="6" t="inlineStr">
+        <x:is>
+          <x:t>lmZaxYlDlkm8GvAK</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H15" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="6"/>
-      <x:c r="B16" s="6"/>
-      <x:c r="C16" s="6"/>
+      <x:c r="A16" s="6" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B16" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D16" s="11"/>
       <x:c r="E16" s="6"/>
-      <x:c r="F16" s="20"/>
-      <x:c r="G16" s="6"/>
-      <x:c r="H16" s="6"/>
+      <x:c r="F16" s="20" t="n">
+        <x:v>0.09783600040728753</x:v>
+      </x:c>
+      <x:c r="G16" s="6" t="inlineStr">
+        <x:is>
+          <x:t>TURANa5f21AmhiAL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H16" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="6"/>
-      <x:c r="B17" s="6"/>
-      <x:c r="C17" s="6"/>
+      <x:c r="A17" s="6" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B17" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D17" s="11"/>
       <x:c r="E17" s="6"/>
-      <x:c r="F17" s="20"/>
-      <x:c r="G17" s="6"/>
-      <x:c r="H17" s="6"/>
+      <x:c r="F17" s="20" t="n">
+        <x:v>0.01182483322098554</x:v>
+      </x:c>
+      <x:c r="G17" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Lvfb3oPsBWLkd53U</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H17" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="6"/>
-      <x:c r="B18" s="6"/>
-      <x:c r="C18" s="6"/>
+      <x:c r="A18" s="6" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B18" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D18" s="11"/>
       <x:c r="E18" s="6"/>
-      <x:c r="F18" s="20"/>
-      <x:c r="G18" s="6"/>
-      <x:c r="H18" s="6"/>
+      <x:c r="F18" s="20" t="n">
+        <x:v>0.005508891622570049</x:v>
+      </x:c>
+      <x:c r="G18" s="6" t="inlineStr">
+        <x:is>
+          <x:t>h5ruIRgO3xgx8u0e</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H18" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="6"/>
-      <x:c r="B19" s="6"/>
-      <x:c r="C19" s="6"/>
+      <x:c r="A19" s="6" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B19" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C19" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D19" s="11"/>
       <x:c r="E19" s="6"/>
-      <x:c r="F19" s="20"/>
-      <x:c r="G19" s="6"/>
-      <x:c r="H19" s="6"/>
+      <x:c r="F19" s="20" t="n">
+        <x:v>0.008159409224324697</x:v>
+      </x:c>
+      <x:c r="G19" s="6" t="inlineStr">
+        <x:is>
+          <x:t>fWCNz2PXNHvUFWzb</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H19" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="6"/>
-      <x:c r="B20" s="6"/>
-      <x:c r="C20" s="6"/>
+      <x:c r="A20" s="6" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B20" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C20" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D20" s="11"/>
       <x:c r="E20" s="6"/>
-      <x:c r="F20" s="20"/>
-      <x:c r="G20" s="6"/>
-      <x:c r="H20" s="6"/>
+      <x:c r="F20" s="20" t="n">
+        <x:v>0.0025197796121315223</x:v>
+      </x:c>
+      <x:c r="G20" s="6" t="inlineStr">
+        <x:is>
+          <x:t>GqUmky5VKcbmgZSU</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H20" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
+      <x:c r="A21" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B21" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C21" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D21" s="23"/>
-      <x:c r="F21" s="24"/>
+      <x:c r="E21"/>
+      <x:c r="F21" s="24" t="n">
+        <x:v>-0.007996728053536637</x:v>
+      </x:c>
+      <x:c r="G21" t="inlineStr">
+        <x:is>
+          <x:t>uTbcKbXAp9Be7SC9</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H21" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
+      <x:c r="A22" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B22" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C22" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D22" s="23"/>
-      <x:c r="F22" s="24"/>
+      <x:c r="E22"/>
+      <x:c r="F22" s="24" t="n">
+        <x:v>0.003354142620959191</x:v>
+      </x:c>
+      <x:c r="G22" t="inlineStr">
+        <x:is>
+          <x:t>dropIGgQmgDH1WRr</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H22" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
+      <x:c r="A23" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B23" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C23" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D23" s="23"/>
-      <x:c r="F23" s="24"/>
+      <x:c r="E23"/>
+      <x:c r="F23" s="24" t="n">
+        <x:v>-0.003039324632075378</x:v>
+      </x:c>
+      <x:c r="G23" t="inlineStr">
+        <x:is>
+          <x:t>uHuan3UDZEwjgWRu</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H23" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
+      <x:c r="A24" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B24" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C24" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D24" s="23"/>
-      <x:c r="F24" s="24"/>
+      <x:c r="E24"/>
+      <x:c r="F24" s="24" t="n">
+        <x:v>0.003992926128141634</x:v>
+      </x:c>
+      <x:c r="G24" t="inlineStr">
+        <x:is>
+          <x:t>J39oxXYGLTa6MPT1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H24" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
+      <x:c r="A25" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B25" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D25" s="23"/>
-      <x:c r="F25" s="24"/>
+      <x:c r="E25"/>
+      <x:c r="F25" s="24" t="n">
+        <x:v>0.001410532636441672</x:v>
+      </x:c>
+      <x:c r="G25" t="inlineStr">
+        <x:is>
+          <x:t>DYdh0YzyFmb55Kqa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H25" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
+      <x:c r="A26" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B26" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C26" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D26" s="23"/>
-      <x:c r="F26" s="24"/>
+      <x:c r="E26"/>
+      <x:c r="F26" s="24" t="n">
+        <x:v>0.010821837995222261</x:v>
+      </x:c>
+      <x:c r="G26" t="inlineStr">
+        <x:is>
+          <x:t>tJKiGWUPHuIzDVo5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H26" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
+      <x:c r="A27" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B27" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C27" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D27" s="23"/>
-      <x:c r="F27" s="24"/>
+      <x:c r="E27"/>
+      <x:c r="F27" s="24" t="n">
+        <x:v>0.004137638963341837</x:v>
+      </x:c>
+      <x:c r="G27" t="inlineStr">
+        <x:is>
+          <x:t>rmB9Wk7PnVRh4Ksr</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H27" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
+      <x:c r="A28" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B28" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C28" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D28" s="23"/>
-      <x:c r="F28" s="24"/>
+      <x:c r="E28"/>
+      <x:c r="F28" s="24" t="n">
+        <x:v>0.01005901714493289</x:v>
+      </x:c>
+      <x:c r="G28" t="inlineStr">
+        <x:is>
+          <x:t>yC1WtwWAmvioU2zI</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H28" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
+      <x:c r="A29" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B29" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C29" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D29" s="23"/>
-      <x:c r="F29" s="24"/>
+      <x:c r="E29"/>
+      <x:c r="F29" s="24" t="n">
+        <x:v>0.013567060511906277</x:v>
+      </x:c>
+      <x:c r="G29" t="inlineStr">
+        <x:is>
+          <x:t>60NGWyMyT4P4BpBG</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H29" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
+      <x:c r="A30" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B30" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C30" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D30" s="23"/>
-      <x:c r="F30" s="24"/>
+      <x:c r="E30"/>
+      <x:c r="F30" s="24" t="n">
+        <x:v>0.007772620923951442</x:v>
+      </x:c>
+      <x:c r="G30" t="inlineStr">
+        <x:is>
+          <x:t>jTnEzaXlM9lrFr9r</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H30" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
+      <x:c r="A31" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B31" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C31" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D31" s="23"/>
-      <x:c r="F31" s="24"/>
+      <x:c r="E31"/>
+      <x:c r="F31" s="24" t="n">
+        <x:v>0.027055551439344877</x:v>
+      </x:c>
+      <x:c r="G31" t="inlineStr">
+        <x:is>
+          <x:t>X314hDD7f4Gk5fD3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H31" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
+      <x:c r="A32" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B32" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C32" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D32" s="23"/>
-      <x:c r="F32" s="24"/>
+      <x:c r="E32"/>
+      <x:c r="F32" s="24" t="n">
+        <x:v>0.05545869149013874</x:v>
+      </x:c>
+      <x:c r="G32" t="inlineStr">
+        <x:is>
+          <x:t>H25PAmPtNUI4jMSY</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H32" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
+      <x:c r="A33" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B33" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C33" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D33" s="23"/>
-      <x:c r="F33" s="24"/>
+      <x:c r="E33"/>
+      <x:c r="F33" s="24" t="n">
+        <x:v>-0.12351751061312799</x:v>
+      </x:c>
+      <x:c r="G33" t="inlineStr">
+        <x:is>
+          <x:t>v1nXgToXExYbkaYq</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H33" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
+      <x:c r="A34" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B34" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C34" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D34" s="23"/>
-      <x:c r="F34" s="24"/>
+      <x:c r="E34"/>
+      <x:c r="F34" s="24" t="n">
+        <x:v>-0.023178016601034756</x:v>
+      </x:c>
+      <x:c r="G34" t="inlineStr">
+        <x:is>
+          <x:t>wlqjcFqMohlSJpSZ</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H34" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
+      <x:c r="A35" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B35" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C35" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D35" s="23"/>
-      <x:c r="F35" s="24"/>
+      <x:c r="E35"/>
+      <x:c r="F35" s="24" t="n">
+        <x:v>0.31045798060214</x:v>
+      </x:c>
+      <x:c r="G35" t="inlineStr">
+        <x:is>
+          <x:t>HCw4rhIo6MdQG7IB</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H35" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
+      <x:c r="A36" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B36" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C36" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D36" s="23"/>
-      <x:c r="F36" s="24"/>
+      <x:c r="E36"/>
+      <x:c r="F36" s="24" t="n">
+        <x:v>0.2833101823456115</x:v>
+      </x:c>
+      <x:c r="G36" t="inlineStr">
+        <x:is>
+          <x:t>xIu0agPgzLMMYLfT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H36" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
+      <x:c r="A37" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B37" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C37" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D37" s="23"/>
-      <x:c r="F37" s="24"/>
+      <x:c r="E37"/>
+      <x:c r="F37" s="24" t="n">
+        <x:v>0.8501876361510272</x:v>
+      </x:c>
+      <x:c r="G37" t="inlineStr">
+        <x:is>
+          <x:t>cH98ezz3SBhTP5mN</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H37" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
+      <x:c r="A38" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B38" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C38" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D38" s="23"/>
-      <x:c r="F38" s="24"/>
+      <x:c r="E38"/>
+      <x:c r="F38" s="24" t="n">
+        <x:v>0.7850472068404161</x:v>
+      </x:c>
+      <x:c r="G38" t="inlineStr">
+        <x:is>
+          <x:t>OIOwNPNfE2loWT37</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H38" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
+      <x:c r="A39" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B39" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C39" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D39" s="23"/>
-      <x:c r="F39" s="24"/>
+      <x:c r="E39"/>
+      <x:c r="F39" s="24" t="n">
+        <x:v>0.993641530105535</x:v>
+      </x:c>
+      <x:c r="G39" t="inlineStr">
+        <x:is>
+          <x:t>8u8qRRzfTbTUBL0R</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H39" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
+      <x:c r="A40" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B40" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C40" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D40" s="23"/>
-      <x:c r="F40" s="24"/>
+      <x:c r="E40"/>
+      <x:c r="F40" s="24" t="n">
+        <x:v>0.9926930178583128</x:v>
+      </x:c>
+      <x:c r="G40" t="inlineStr">
+        <x:is>
+          <x:t>Wsto0FWElr5r0r5i</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H40" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
+      <x:c r="A41" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B41" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C41" t="n">
+        <x:v>256</x:v>
+      </x:c>
       <x:c r="D41" s="23"/>
-      <x:c r="F41" s="24"/>
+      <x:c r="E41"/>
+      <x:c r="F41" s="24" t="n">
+        <x:v>0.9913355692134291</x:v>
+      </x:c>
+      <x:c r="G41" t="inlineStr">
+        <x:is>
+          <x:t>5dZ0YweCedhtfDwr</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H41" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="42">
+      <x:c r="A42" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B42" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C42" t="n">
+        <x:v>256</x:v>
+      </x:c>
       <x:c r="D42" s="23"/>
-      <x:c r="F42" s="24"/>
+      <x:c r="E42"/>
+      <x:c r="F42" s="24" t="n">
+        <x:v>0.9809161032568489</x:v>
+      </x:c>
+      <x:c r="G42" t="inlineStr">
+        <x:is>
+          <x:t>s3cfGVuRsQgsdzja</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H42" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
+      <x:c r="A43" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B43" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C43" t="n">
+        <x:v>256</x:v>
+      </x:c>
       <x:c r="D43" s="23"/>
-      <x:c r="F43" s="24"/>
+      <x:c r="E43"/>
+      <x:c r="F43" s="24" t="n">
+        <x:v>0.8540493001985443</x:v>
+      </x:c>
+      <x:c r="G43" t="inlineStr">
+        <x:is>
+          <x:t>R8m8vWL7bqHwjZ8z</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H43" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="D44" s="23"/>
@@ -18370,311 +19211,1408 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="6"/>
-      <x:c r="B5" s="6"/>
-      <x:c r="C5" s="6"/>
+      <x:c r="A5" s="6" t="inlineStr">
+        <x:is>
+          <x:t>3vthFykOUg9STpyH</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B5" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C5" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D5" s="11"/>
       <x:c r="E5" s="6"/>
-      <x:c r="F5" s="6"/>
-      <x:c r="G5" s="6"/>
-      <x:c r="H5" s="7"/>
-      <x:c r="I5" s="7"/>
-      <x:c r="J5" s="6"/>
+      <x:c r="F5" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G5" s="6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H5" s="7" t="n">
+        <x:v>91.811</x:v>
+      </x:c>
+      <x:c r="I5" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J5" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 052f669dc83a7ac6ca45</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="6"/>
-      <x:c r="B6" s="6"/>
-      <x:c r="C6" s="6"/>
+      <x:c r="A6" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Yxrh3L2PUkc3VhaY</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B6" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C6" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D6" s="11"/>
       <x:c r="E6" s="6"/>
-      <x:c r="F6" s="6"/>
-      <x:c r="G6" s="6"/>
-      <x:c r="H6" s="7"/>
-      <x:c r="I6" s="7"/>
-      <x:c r="J6" s="6"/>
+      <x:c r="F6" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G6" s="6" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H6" s="7" t="n">
+        <x:v>68.077</x:v>
+      </x:c>
+      <x:c r="I6" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J6" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 362080c421bc65f1b51f</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="6"/>
-      <x:c r="B7" s="6"/>
-      <x:c r="C7" s="6"/>
+      <x:c r="A7" s="6" t="inlineStr">
+        <x:is>
+          <x:t>amYn6eEGELs0f07u</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B7" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C7" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D7" s="11"/>
       <x:c r="E7" s="6"/>
-      <x:c r="F7" s="6"/>
-      <x:c r="G7" s="6"/>
-      <x:c r="H7" s="7"/>
-      <x:c r="I7" s="7"/>
-      <x:c r="J7" s="6"/>
+      <x:c r="F7" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G7" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H7" s="7" t="n">
+        <x:v>93.863</x:v>
+      </x:c>
+      <x:c r="I7" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J7" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 038dae412b43db850131</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="6"/>
-      <x:c r="B8" s="6"/>
-      <x:c r="C8" s="6"/>
+      <x:c r="A8" s="6" t="inlineStr">
+        <x:is>
+          <x:t>CcP073uy8VTfOm7Z</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B8" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C8" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D8" s="11"/>
       <x:c r="E8" s="6"/>
-      <x:c r="F8" s="6"/>
-      <x:c r="G8" s="6"/>
-      <x:c r="H8" s="7"/>
-      <x:c r="I8" s="7"/>
-      <x:c r="J8" s="6"/>
+      <x:c r="F8" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G8" s="6" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H8" s="7" t="n">
+        <x:v>101.714</x:v>
+      </x:c>
+      <x:c r="I8" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J8" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 5a98c6e2083a74cd5901</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="6"/>
-      <x:c r="B9" s="6"/>
-      <x:c r="C9" s="6"/>
+      <x:c r="A9" s="6" t="inlineStr">
+        <x:is>
+          <x:t>naxElkaIO19i9Z0B</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B9" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C9" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D9" s="11"/>
       <x:c r="E9" s="6"/>
-      <x:c r="F9" s="6"/>
-      <x:c r="G9" s="6"/>
-      <x:c r="H9" s="7"/>
-      <x:c r="I9" s="7"/>
-      <x:c r="J9" s="6"/>
+      <x:c r="F9" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G9" s="6" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H9" s="7" t="n">
+        <x:v>96.882</x:v>
+      </x:c>
+      <x:c r="I9" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J9" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 6b7d603e7cd2c913101a</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="6"/>
-      <x:c r="B10" s="6"/>
-      <x:c r="C10" s="6"/>
+      <x:c r="A10" s="6" t="inlineStr">
+        <x:is>
+          <x:t>culHIrNwFvzVmhin</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B10" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C10" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D10" s="11"/>
       <x:c r="E10" s="6"/>
-      <x:c r="F10" s="6"/>
-      <x:c r="G10" s="6"/>
-      <x:c r="H10" s="7"/>
-      <x:c r="I10" s="7"/>
-      <x:c r="J10" s="6"/>
+      <x:c r="F10" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G10" s="6" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H10" s="7" t="n">
+        <x:v>110.247</x:v>
+      </x:c>
+      <x:c r="I10" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J10" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner cf699dcf18deac2218e3</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="6"/>
-      <x:c r="B11" s="6"/>
-      <x:c r="C11" s="6"/>
+      <x:c r="A11" s="6" t="inlineStr">
+        <x:is>
+          <x:t>B4ds8Aiw7rfVMwe3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B11" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C11" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D11" s="11"/>
       <x:c r="E11" s="6"/>
-      <x:c r="F11" s="6"/>
-      <x:c r="G11" s="6"/>
-      <x:c r="H11" s="7"/>
-      <x:c r="I11" s="7"/>
-      <x:c r="J11" s="6"/>
+      <x:c r="F11" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G11" s="6" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H11" s="7" t="n">
+        <x:v>121.203</x:v>
+      </x:c>
+      <x:c r="I11" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J11" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 241879f0a1ec3ba03aad</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="6"/>
-      <x:c r="B12" s="6"/>
-      <x:c r="C12" s="6"/>
+      <x:c r="A12" s="6" t="inlineStr">
+        <x:is>
+          <x:t>cMCDoXnvsIcrGYIL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B12" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D12" s="11"/>
       <x:c r="E12" s="6"/>
-      <x:c r="F12" s="6"/>
-      <x:c r="G12" s="6"/>
-      <x:c r="H12" s="7"/>
-      <x:c r="I12" s="7"/>
-      <x:c r="J12" s="6"/>
+      <x:c r="F12" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G12" s="6" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H12" s="7" t="n">
+        <x:v>104.168</x:v>
+      </x:c>
+      <x:c r="I12" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J12" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner d1024a5d898d01edec79</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="6"/>
-      <x:c r="B13" s="6"/>
-      <x:c r="C13" s="6"/>
+      <x:c r="A13" s="6" t="inlineStr">
+        <x:is>
+          <x:t>iqlVmKsTe1h6oCoX</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B13" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C13" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D13" s="11"/>
       <x:c r="E13" s="6"/>
-      <x:c r="F13" s="6"/>
-      <x:c r="G13" s="6"/>
-      <x:c r="H13" s="7"/>
-      <x:c r="I13" s="7"/>
-      <x:c r="J13" s="6"/>
+      <x:c r="F13" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G13" s="6" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H13" s="7" t="n">
+        <x:v>90.268</x:v>
+      </x:c>
+      <x:c r="I13" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J13" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 2913e9c5811a9389b80c</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="6"/>
-      <x:c r="B14" s="6"/>
-      <x:c r="C14" s="6"/>
+      <x:c r="A14" s="6" t="inlineStr">
+        <x:is>
+          <x:t>ddxYjwvqBs0JhZtJ</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B14" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D14" s="11"/>
       <x:c r="E14" s="6"/>
-      <x:c r="F14" s="6"/>
-      <x:c r="G14" s="6"/>
-      <x:c r="H14" s="7"/>
-      <x:c r="I14" s="7"/>
-      <x:c r="J14" s="6"/>
+      <x:c r="F14" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G14" s="6" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H14" s="7" t="n">
+        <x:v>91.759</x:v>
+      </x:c>
+      <x:c r="I14" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J14" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 4e0b980e893e9a071027</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="6"/>
-      <x:c r="B15" s="6"/>
-      <x:c r="C15" s="6"/>
+      <x:c r="A15" s="6" t="inlineStr">
+        <x:is>
+          <x:t>lmZaxYlDlkm8GvAK</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B15" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C15" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D15" s="11"/>
       <x:c r="E15" s="6"/>
-      <x:c r="F15" s="6"/>
-      <x:c r="G15" s="6"/>
-      <x:c r="H15" s="7"/>
-      <x:c r="I15" s="7"/>
-      <x:c r="J15" s="6"/>
+      <x:c r="F15" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G15" s="6" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H15" s="7" t="n">
+        <x:v>114.056</x:v>
+      </x:c>
+      <x:c r="I15" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J15" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 9ce660a0ed78d8defa95</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="6"/>
-      <x:c r="B16" s="6"/>
-      <x:c r="C16" s="6"/>
+      <x:c r="A16" s="6" t="inlineStr">
+        <x:is>
+          <x:t>TURANa5f21AmhiAL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B16" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D16" s="11"/>
       <x:c r="E16" s="6"/>
-      <x:c r="F16" s="6"/>
-      <x:c r="G16" s="6"/>
-      <x:c r="H16" s="7"/>
-      <x:c r="I16" s="7"/>
-      <x:c r="J16" s="6"/>
+      <x:c r="F16" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G16" s="6" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H16" s="7" t="n">
+        <x:v>94.176</x:v>
+      </x:c>
+      <x:c r="I16" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J16" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner f82fd27456b62ea723ca</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="6"/>
-      <x:c r="B17" s="6"/>
-      <x:c r="C17" s="6"/>
+      <x:c r="A17" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Lvfb3oPsBWLkd53U</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B17" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D17" s="11"/>
       <x:c r="E17" s="6"/>
-      <x:c r="F17" s="6"/>
-      <x:c r="G17" s="6"/>
-      <x:c r="H17" s="7"/>
-      <x:c r="I17" s="7"/>
-      <x:c r="J17" s="6"/>
+      <x:c r="F17" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G17" s="6" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H17" s="7" t="n">
+        <x:v>98.661</x:v>
+      </x:c>
+      <x:c r="I17" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J17" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 9b7859cdebd9e0e41eee</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="6"/>
-      <x:c r="B18" s="6"/>
-      <x:c r="C18" s="6"/>
+      <x:c r="A18" s="6" t="inlineStr">
+        <x:is>
+          <x:t>h5ruIRgO3xgx8u0e</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B18" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D18" s="11"/>
       <x:c r="E18" s="6"/>
-      <x:c r="F18" s="6"/>
-      <x:c r="G18" s="6"/>
-      <x:c r="H18" s="7"/>
-      <x:c r="I18" s="7"/>
-      <x:c r="J18" s="6"/>
+      <x:c r="F18" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G18" s="6" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H18" s="7" t="n">
+        <x:v>122.872</x:v>
+      </x:c>
+      <x:c r="I18" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J18" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner a80def0e6379bb520937</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="6"/>
-      <x:c r="B19" s="6"/>
-      <x:c r="C19" s="6"/>
+      <x:c r="A19" s="6" t="inlineStr">
+        <x:is>
+          <x:t>fWCNz2PXNHvUFWzb</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B19" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C19" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D19" s="11"/>
       <x:c r="E19" s="6"/>
-      <x:c r="F19" s="6"/>
-      <x:c r="G19" s="6"/>
-      <x:c r="H19" s="7"/>
-      <x:c r="I19" s="7"/>
-      <x:c r="J19" s="6"/>
+      <x:c r="F19" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G19" s="6" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H19" s="7" t="n">
+        <x:v>124.812</x:v>
+      </x:c>
+      <x:c r="I19" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J19" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner 821edd467bf428427e4a</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="6"/>
-      <x:c r="B20" s="6"/>
-      <x:c r="C20" s="6"/>
+      <x:c r="A20" s="6" t="inlineStr">
+        <x:is>
+          <x:t>GqUmky5VKcbmgZSU</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B20" s="6" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C20" s="6" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D20" s="11"/>
       <x:c r="E20" s="6"/>
-      <x:c r="F20" s="6"/>
-      <x:c r="G20" s="6"/>
-      <x:c r="H20" s="7"/>
-      <x:c r="I20" s="7"/>
-      <x:c r="J20" s="6"/>
+      <x:c r="F20" s="6" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G20" s="6" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H20" s="7" t="n">
+        <x:v>135.492</x:v>
+      </x:c>
+      <x:c r="I20" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J20" s="6" t="inlineStr">
+        <x:is>
+          <x:t>runner f79961a19db100f1d7e4</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="21">
+      <x:c r="A21" t="inlineStr">
+        <x:is>
+          <x:t>uTbcKbXAp9Be7SC9</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B21" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C21" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D21" s="23"/>
-      <x:c r="H21" s="25"/>
-      <x:c r="I21" s="25"/>
+      <x:c r="E21"/>
+      <x:c r="F21" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G21" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H21" s="25" t="n">
+        <x:v>112.531</x:v>
+      </x:c>
+      <x:c r="I21" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J21" t="inlineStr">
+        <x:is>
+          <x:t>runner 0b7e3393769d8e1d1055</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="22">
+      <x:c r="A22" t="inlineStr">
+        <x:is>
+          <x:t>dropIGgQmgDH1WRr</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B22" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C22" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D22" s="23"/>
-      <x:c r="H22" s="25"/>
-      <x:c r="I22" s="25"/>
+      <x:c r="E22"/>
+      <x:c r="F22" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G22" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H22" s="25" t="n">
+        <x:v>101.693</x:v>
+      </x:c>
+      <x:c r="I22" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J22" t="inlineStr">
+        <x:is>
+          <x:t>runner a3f91e55bf33b0162870</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="23">
+      <x:c r="A23" t="inlineStr">
+        <x:is>
+          <x:t>uHuan3UDZEwjgWRu</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B23" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C23" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D23" s="23"/>
-      <x:c r="H23" s="25"/>
-      <x:c r="I23" s="25"/>
+      <x:c r="E23"/>
+      <x:c r="F23" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G23" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="H23" s="25" t="n">
+        <x:v>129.099</x:v>
+      </x:c>
+      <x:c r="I23" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J23" t="inlineStr">
+        <x:is>
+          <x:t>runner daf688c12a10ef8579e8</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="24">
+      <x:c r="A24" t="inlineStr">
+        <x:is>
+          <x:t>J39oxXYGLTa6MPT1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B24" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C24" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D24" s="23"/>
-      <x:c r="H24" s="25"/>
-      <x:c r="I24" s="25"/>
+      <x:c r="E24"/>
+      <x:c r="F24" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G24" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="H24" s="25" t="n">
+        <x:v>127.835</x:v>
+      </x:c>
+      <x:c r="I24" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J24" t="inlineStr">
+        <x:is>
+          <x:t>runner 41b1ad8a5cf3ca9cd551</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="25">
+      <x:c r="A25" t="inlineStr">
+        <x:is>
+          <x:t>DYdh0YzyFmb55Kqa</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B25" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D25" s="23"/>
-      <x:c r="H25" s="25"/>
-      <x:c r="I25" s="25"/>
+      <x:c r="E25"/>
+      <x:c r="F25" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G25" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H25" s="25" t="n">
+        <x:v>126.932</x:v>
+      </x:c>
+      <x:c r="I25" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J25" t="inlineStr">
+        <x:is>
+          <x:t>runner 4c323cfb55502d99b628</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="26">
+      <x:c r="A26" t="inlineStr">
+        <x:is>
+          <x:t>tJKiGWUPHuIzDVo5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B26" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C26" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D26" s="23"/>
-      <x:c r="H26" s="25"/>
-      <x:c r="I26" s="25"/>
+      <x:c r="E26"/>
+      <x:c r="F26" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G26" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="H26" s="25" t="n">
+        <x:v>99.94</x:v>
+      </x:c>
+      <x:c r="I26" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J26" t="inlineStr">
+        <x:is>
+          <x:t>runner b6aaf8508e818eca6d5c</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="27">
+      <x:c r="A27" t="inlineStr">
+        <x:is>
+          <x:t>rmB9Wk7PnVRh4Ksr</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B27" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C27" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D27" s="23"/>
-      <x:c r="H27" s="25"/>
-      <x:c r="I27" s="25"/>
+      <x:c r="E27"/>
+      <x:c r="F27" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G27" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H27" s="25" t="n">
+        <x:v>136.785</x:v>
+      </x:c>
+      <x:c r="I27" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J27" t="inlineStr">
+        <x:is>
+          <x:t>runner c5ea3ec8d23b93758e6d</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="28">
+      <x:c r="A28" t="inlineStr">
+        <x:is>
+          <x:t>yC1WtwWAmvioU2zI</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B28" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C28" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D28" s="23"/>
-      <x:c r="H28" s="25"/>
-      <x:c r="I28" s="25"/>
+      <x:c r="E28"/>
+      <x:c r="F28" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G28" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="H28" s="25" t="n">
+        <x:v>137.351</x:v>
+      </x:c>
+      <x:c r="I28" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J28" t="inlineStr">
+        <x:is>
+          <x:t>runner fd2bfcd353bac27a1cd5</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="29">
+      <x:c r="A29" t="inlineStr">
+        <x:is>
+          <x:t>60NGWyMyT4P4BpBG</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B29" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C29" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D29" s="23"/>
-      <x:c r="H29" s="25"/>
-      <x:c r="I29" s="25"/>
+      <x:c r="E29"/>
+      <x:c r="F29" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G29" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="H29" s="25" t="n">
+        <x:v>136.045</x:v>
+      </x:c>
+      <x:c r="I29" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J29" t="inlineStr">
+        <x:is>
+          <x:t>runner 1d420e487ebdcf9ff33e</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="30">
+      <x:c r="A30" t="inlineStr">
+        <x:is>
+          <x:t>jTnEzaXlM9lrFr9r</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B30" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C30" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D30" s="23"/>
-      <x:c r="H30" s="25"/>
-      <x:c r="I30" s="25"/>
+      <x:c r="E30"/>
+      <x:c r="F30" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G30" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="H30" s="25" t="n">
+        <x:v>118.86</x:v>
+      </x:c>
+      <x:c r="I30" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J30" t="inlineStr">
+        <x:is>
+          <x:t>runner 1a77d8bbb214b0ac3cfb</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="31">
+      <x:c r="A31" t="inlineStr">
+        <x:is>
+          <x:t>X314hDD7f4Gk5fD3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B31" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C31" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D31" s="23"/>
-      <x:c r="H31" s="25"/>
-      <x:c r="I31" s="25"/>
+      <x:c r="E31"/>
+      <x:c r="F31" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G31" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="H31" s="25" t="n">
+        <x:v>101.058</x:v>
+      </x:c>
+      <x:c r="I31" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J31" t="inlineStr">
+        <x:is>
+          <x:t>runner 4d223b034e139f87c35a</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="32">
+      <x:c r="A32" t="inlineStr">
+        <x:is>
+          <x:t>H25PAmPtNUI4jMSY</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B32" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C32" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D32" s="23"/>
-      <x:c r="H32" s="25"/>
-      <x:c r="I32" s="25"/>
+      <x:c r="E32"/>
+      <x:c r="F32" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G32" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="H32" s="25" t="n">
+        <x:v>126.077</x:v>
+      </x:c>
+      <x:c r="I32" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J32" t="inlineStr">
+        <x:is>
+          <x:t>runner b1a47beee276ac3601dd</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="33">
+      <x:c r="A33" t="inlineStr">
+        <x:is>
+          <x:t>v1nXgToXExYbkaYq</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B33" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C33" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D33" s="23"/>
-      <x:c r="H33" s="25"/>
-      <x:c r="I33" s="25"/>
+      <x:c r="E33"/>
+      <x:c r="F33" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G33" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="H33" s="25" t="n">
+        <x:v>99.766</x:v>
+      </x:c>
+      <x:c r="I33" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J33" t="inlineStr">
+        <x:is>
+          <x:t>runner e01029f4920f043c0b6f</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="34">
+      <x:c r="A34" t="inlineStr">
+        <x:is>
+          <x:t>wlqjcFqMohlSJpSZ</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B34" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C34" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D34" s="23"/>
-      <x:c r="H34" s="25"/>
-      <x:c r="I34" s="25"/>
+      <x:c r="E34"/>
+      <x:c r="F34" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G34" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="H34" s="25" t="n">
+        <x:v>106.329</x:v>
+      </x:c>
+      <x:c r="I34" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J34" t="inlineStr">
+        <x:is>
+          <x:t>runner dc974af70f516aa410c3</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="35">
+      <x:c r="A35" t="inlineStr">
+        <x:is>
+          <x:t>HCw4rhIo6MdQG7IB</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B35" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C35" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D35" s="23"/>
-      <x:c r="H35" s="25"/>
-      <x:c r="I35" s="25"/>
+      <x:c r="E35"/>
+      <x:c r="F35" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G35" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="H35" s="25" t="n">
+        <x:v>115.452</x:v>
+      </x:c>
+      <x:c r="I35" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J35" t="inlineStr">
+        <x:is>
+          <x:t>runner 3b44efb91dac6b7c1b58</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="36">
+      <x:c r="A36" t="inlineStr">
+        <x:is>
+          <x:t>xIu0agPgzLMMYLfT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B36" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C36" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D36" s="23"/>
-      <x:c r="H36" s="25"/>
-      <x:c r="I36" s="25"/>
+      <x:c r="E36"/>
+      <x:c r="F36" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G36" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="H36" s="25" t="n">
+        <x:v>115.092</x:v>
+      </x:c>
+      <x:c r="I36" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J36" t="inlineStr">
+        <x:is>
+          <x:t>runner 7321963159ab2fc2677f</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="37">
+      <x:c r="A37" t="inlineStr">
+        <x:is>
+          <x:t>cH98ezz3SBhTP5mN</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B37" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C37" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D37" s="23"/>
-      <x:c r="H37" s="25"/>
-      <x:c r="I37" s="25"/>
+      <x:c r="E37"/>
+      <x:c r="F37" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G37" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="H37" s="25" t="n">
+        <x:v>104.631</x:v>
+      </x:c>
+      <x:c r="I37" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J37" t="inlineStr">
+        <x:is>
+          <x:t>runner 9e359d3fc2899473b0ed</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="38">
+      <x:c r="A38" t="inlineStr">
+        <x:is>
+          <x:t>OIOwNPNfE2loWT37</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B38" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C38" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D38" s="23"/>
-      <x:c r="H38" s="25"/>
-      <x:c r="I38" s="25"/>
+      <x:c r="E38"/>
+      <x:c r="F38" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G38" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="H38" s="25" t="n">
+        <x:v>96.639</x:v>
+      </x:c>
+      <x:c r="I38" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J38" t="inlineStr">
+        <x:is>
+          <x:t>runner ec9c888bd9749b283c5b</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="39">
+      <x:c r="A39" t="inlineStr">
+        <x:is>
+          <x:t>8u8qRRzfTbTUBL0R</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B39" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C39" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D39" s="23"/>
-      <x:c r="H39" s="25"/>
-      <x:c r="I39" s="25"/>
+      <x:c r="E39"/>
+      <x:c r="F39" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G39" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="H39" s="25" t="n">
+        <x:v>80.045</x:v>
+      </x:c>
+      <x:c r="I39" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J39" t="inlineStr">
+        <x:is>
+          <x:t>runner c45d5314bb9440d507ac</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="40">
+      <x:c r="A40" t="inlineStr">
+        <x:is>
+          <x:t>Wsto0FWElr5r0r5i</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B40" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C40" t="n">
+        <x:v>128</x:v>
+      </x:c>
       <x:c r="D40" s="23"/>
-      <x:c r="H40" s="25"/>
-      <x:c r="I40" s="25"/>
+      <x:c r="E40"/>
+      <x:c r="F40" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G40" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="H40" s="25" t="n">
+        <x:v>97.178</x:v>
+      </x:c>
+      <x:c r="I40" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J40" t="inlineStr">
+        <x:is>
+          <x:t>runner b343218d6614fe2e9daa</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="41">
+      <x:c r="A41" t="inlineStr">
+        <x:is>
+          <x:t>5dZ0YweCedhtfDwr</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B41" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C41" t="n">
+        <x:v>256</x:v>
+      </x:c>
       <x:c r="D41" s="23"/>
-      <x:c r="H41" s="25"/>
-      <x:c r="I41" s="25"/>
+      <x:c r="E41"/>
+      <x:c r="F41" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G41" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H41" s="25" t="n">
+        <x:v>103.979</x:v>
+      </x:c>
+      <x:c r="I41" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J41" t="inlineStr">
+        <x:is>
+          <x:t>runner 245ce15ea17747b5e730</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="42">
+      <x:c r="A42" t="inlineStr">
+        <x:is>
+          <x:t>s3cfGVuRsQgsdzja</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B42" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C42" t="n">
+        <x:v>256</x:v>
+      </x:c>
       <x:c r="D42" s="23"/>
-      <x:c r="H42" s="25"/>
-      <x:c r="I42" s="25"/>
+      <x:c r="E42"/>
+      <x:c r="F42" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G42" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H42" s="25" t="n">
+        <x:v>98.081</x:v>
+      </x:c>
+      <x:c r="I42" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J42" t="inlineStr">
+        <x:is>
+          <x:t>runner 39a4fecaade4edadfc28</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="43">
+      <x:c r="A43" t="inlineStr">
+        <x:is>
+          <x:t>R8m8vWL7bqHwjZ8z</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B43" t="inlineStr">
+        <x:is>
+          <x:t>MPS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C43" t="n">
+        <x:v>256</x:v>
+      </x:c>
       <x:c r="D43" s="23"/>
-      <x:c r="H43" s="25"/>
-      <x:c r="I43" s="25"/>
+      <x:c r="E43"/>
+      <x:c r="F43" t="inlineStr">
+        <x:is>
+          <x:t>succeeded</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G43" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H43" s="25" t="n">
+        <x:v>97.978</x:v>
+      </x:c>
+      <x:c r="I43" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J43" t="inlineStr">
+        <x:is>
+          <x:t>runner d820da970ec6b1d7df27</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="D44" s="23"/>

</xml_diff>